<commit_message>
Merge project imports by number and support title rows
</commit_message>
<xml_diff>
--- a/Projektinfos_einheitlich_5_bis_12_kapazitaeten_mind1200.xlsx
+++ b/Projektinfos_einheitlich_5_bis_12_kapazitaeten_mind1200.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hendrik\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e014d81cf04334bc/Beruf/Organisatorisches/Workbench/Projektzuordnung/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B10200F0-5B1A-4020-82E2-B6EB30209EB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{B10200F0-5B1A-4020-82E2-B6EB30209EB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47C8A365-A620-4C32-BC68-F6000FF03D1A}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="73">
   <si>
     <t>Projekt-beschreibung</t>
   </si>
@@ -228,6 +228,21 @@
   </si>
   <si>
     <t>Abschlussausstellung aufbauen: Zum Ende der Projektwoche planen und gestalten wir eine Präsentationsfläche für Ergebnisse, Fotos und Werkstücke.</t>
+  </si>
+  <si>
+    <t>5–8</t>
+  </si>
+  <si>
+    <t>6–10</t>
+  </si>
+  <si>
+    <t>5–9</t>
+  </si>
+  <si>
+    <t>7–11</t>
+  </si>
+  <si>
+    <t>5–6, 9-10</t>
   </si>
 </sst>
 </file>
@@ -519,7 +534,7 @@
         <v>30</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>12</v>
+        <v>72</v>
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -541,7 +556,7 @@
         <v>32</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>14</v>
+        <v>68</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -563,7 +578,7 @@
         <v>30</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>16</v>
+        <v>69</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
@@ -585,7 +600,7 @@
         <v>15</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>18</v>
+        <v>70</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -607,7 +622,7 @@
         <v>30</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>20</v>
+        <v>71</v>
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>

</xml_diff>